<commit_message>
work-experience.html and styles.css modified
</commit_message>
<xml_diff>
--- a/Test Plan/Test Plan.xlsx
+++ b/Test Plan/Test Plan.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educwaac-my.sharepoint.com/personal/451102_edu_cwa_ac_uk/Documents/College Work/Assignments/Digital Portfolio/Creation/Test Plan/"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -56,10 +56,10 @@
     <t>Success (Yes/No)</t>
   </si>
   <si>
+    <t>Checking if all links click</t>
+  </si>
+  <si>
     <t>Navigates to every link that is clicked on</t>
-  </si>
-  <si>
-    <t>Checking if all links click</t>
   </si>
   <si>
     <t>Check if website works on all devices under 768px</t>
@@ -76,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -512,7 +512,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1BEF50-4814-4512-A0DE-435D547D7E8D}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="76.28515625" customWidth="1"/>
     <col min="3" max="3" width="45.28515625" customWidth="1"/>
@@ -520,7 +520,7 @@
     <col min="5" max="5" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -537,18 +537,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="70.5" customHeight="1">
       <c r="A2">
         <v>1.1000000000000001</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" ht="340.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="340.5" customHeight="1">
       <c r="A3">
         <v>1.2</v>
       </c>
@@ -562,12 +562,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="65.25" customHeight="1">
       <c r="A4">
         <v>1.3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="55.5" customHeight="1">
       <c r="A5">
         <v>1.4</v>
       </c>

</xml_diff>